<commit_message>
Actualiza estado del plan de 2 semanas segun tablero Trello (2026-10-01)
Sincroniza estados de S1 y S2 en Plan_Trabajo_2_Semanas.md y Plan_Trabajo_Trello_Import.xlsx. 'tambien en desarrollo' se registra como En desarrollo en el plan; el Excel usa los nombres de las listas de Trello.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/documentacion/Plan_Trabajo_Trello_Import.xlsx
+++ b/documentacion/Plan_Trabajo_Trello_Import.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -504,7 +504,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -531,7 +531,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>tambien en desarrollo</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>tambien en desarrollo</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>tambien en desarrollo</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Agrega plan historico de semanas 1 y 2 con estados de Trello (2026-10-01)
Guarda el plan S1/S2 actualizado como Plan_Trabajo_Semanas_1_y_2.md para no pisar el plan vigente de semanas 3 y 4, y actualiza los estados en Plan_Trabajo_Trello_Import.xlsx con los nombres de las listas de Trello.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/documentacion/Plan_Trabajo_Trello_Import.xlsx
+++ b/documentacion/Plan_Trabajo_Trello_Import.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -504,7 +504,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -531,7 +531,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>finalizado</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>tambien en desarrollo</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>tambien en desarrollo</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>tambien en desarrollo</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>por hacer</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">

</xml_diff>